<commit_message>
Admin character and chatbot response update
</commit_message>
<xml_diff>
--- a/relationship_data_template.xlsx
+++ b/relationship_data_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krish\OneDrive\Desktop\anime_ai\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krish\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4723F0A2-C930-42BD-99A3-5D9F2B83CEA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F8AF4E-3941-4D7B-95C0-80C677F644FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1C80641A-8C68-4CCB-904C-C1A2FE90DEC2}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4974" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5092" uniqueCount="384">
   <si>
     <t>source_name</t>
   </si>
@@ -1038,23 +1038,158 @@
     <t>char_smoothie_charlotte</t>
   </si>
   <si>
-    <t>Konohagakure</t>
-  </si>
-  <si>
-    <t>org_konohagakure</t>
+    <t>org_straw_hat_pirates</t>
+  </si>
+  <si>
+    <t>Straw Hat Pirates</t>
+  </si>
+  <si>
+    <t>captain</t>
+  </si>
+  <si>
+    <t>organization</t>
+  </si>
+  <si>
+    <t>Zoro Roronoa</t>
+  </si>
+  <si>
+    <t>char_zoro_roronoa</t>
+  </si>
+  <si>
+    <t>Nami</t>
+  </si>
+  <si>
+    <t>char_nami</t>
+  </si>
+  <si>
+    <t>Franky</t>
+  </si>
+  <si>
+    <t>char_franky</t>
+  </si>
+  <si>
+    <t>Brook</t>
+  </si>
+  <si>
+    <t>char_brook</t>
+  </si>
+  <si>
+    <t>Chopper Tony Tony</t>
+  </si>
+  <si>
+    <t>char_chopper_tony_tony</t>
+  </si>
+  <si>
+    <t>vice_captain</t>
   </si>
   <si>
     <t>member</t>
   </si>
   <si>
-    <t>organization</t>
+    <t xml:space="preserve">Captain </t>
+  </si>
+  <si>
+    <t>Swordsman, 3 swords user</t>
+  </si>
+  <si>
+    <t>Navigator</t>
+  </si>
+  <si>
+    <t>Sniper</t>
+  </si>
+  <si>
+    <t>Cook</t>
+  </si>
+  <si>
+    <t>Shipwrighter</t>
+  </si>
+  <si>
+    <t>Doctor</t>
+  </si>
+  <si>
+    <t>Archeologist</t>
+  </si>
+  <si>
+    <t>Singer</t>
+  </si>
+  <si>
+    <t>char_jinbe</t>
+  </si>
+  <si>
+    <t>Jinbe</t>
+  </si>
+  <si>
+    <t>fishman</t>
+  </si>
+  <si>
+    <t>Survey Corps</t>
+  </si>
+  <si>
+    <t>org_survey_corps</t>
+  </si>
+  <si>
+    <t>Erwin Smith</t>
+  </si>
+  <si>
+    <t>char_erwin_smith</t>
+  </si>
+  <si>
+    <t>commander</t>
+  </si>
+  <si>
+    <t>Levi</t>
+  </si>
+  <si>
+    <t>char_levi</t>
+  </si>
+  <si>
+    <t>Captain of the Levi squad</t>
+  </si>
+  <si>
+    <t>Member of the levi squad</t>
+  </si>
+  <si>
+    <t>Mikasa Ackerman</t>
+  </si>
+  <si>
+    <t>char_mikasa_ackerman</t>
+  </si>
+  <si>
+    <t>Armin Arlert</t>
+  </si>
+  <si>
+    <t>char_armin_arlert</t>
+  </si>
+  <si>
+    <t>Hange Zoe</t>
+  </si>
+  <si>
+    <t>char_hange_zoe</t>
+  </si>
+  <si>
+    <t>Jean Kirstein</t>
+  </si>
+  <si>
+    <t>char_jean_kirstein</t>
+  </si>
+  <si>
+    <t>Connie Springer</t>
+  </si>
+  <si>
+    <t>char_connie_springer</t>
+  </si>
+  <si>
+    <t>Sasha Blouse</t>
+  </si>
+  <si>
+    <t>char_sasha_blouse</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1212,6 +1347,30 @@
       <sz val="7"/>
       <color rgb="FF12824D"/>
       <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFA2FCA2"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFCE9178"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFA2FCA2"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFA2FCA2"/>
+      <name val="Consolas"/>
       <family val="3"/>
     </font>
   </fonts>
@@ -1556,7 +1715,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1564,6 +1723,18 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1919,16 +2090,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1F906C6-76EC-4EFB-AFDE-921EF73AD1B4}">
-  <dimension ref="A1:H822"/>
+  <dimension ref="A1:H839"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" customWidth="1"/>
-    <col min="4" max="4" width="27.77734375" customWidth="1"/>
+    <col min="3" max="3" width="23.33203125" customWidth="1"/>
+    <col min="4" max="4" width="37.88671875" customWidth="1"/>
     <col min="5" max="5" width="17.88671875" customWidth="1"/>
     <col min="6" max="6" width="16.6640625" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="7" max="7" width="24.88671875" customWidth="1"/>
     <col min="8" max="8" width="19.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -18280,32 +18451,420 @@
         <v>63</v>
       </c>
     </row>
-    <row r="821" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="820" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A820" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="B820" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="C820" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D820" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E820" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="F820" t="s">
+        <v>338</v>
+      </c>
+      <c r="G820" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="821" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A821" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="B821" t="s">
         <v>335</v>
       </c>
-      <c r="B821" s="4" t="s">
-        <v>336</v>
-      </c>
-      <c r="C821" t="s">
-        <v>8</v>
-      </c>
-      <c r="D821" t="s">
-        <v>9</v>
-      </c>
-      <c r="E821" t="s">
-        <v>337</v>
+      <c r="C821" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="D821" s="7" t="s">
+        <v>340</v>
+      </c>
+      <c r="E821" s="6" t="s">
+        <v>349</v>
       </c>
       <c r="F821" t="s">
         <v>338</v>
       </c>
-    </row>
-    <row r="822" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G821" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="822" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A822" t="s">
+        <v>336</v>
+      </c>
+      <c r="B822" t="s">
         <v>335</v>
       </c>
-      <c r="B822" t="s">
+      <c r="C822" s="7" t="s">
+        <v>341</v>
+      </c>
+      <c r="D822" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="E822" t="s">
+        <v>350</v>
+      </c>
+      <c r="F822" t="s">
+        <v>338</v>
+      </c>
+      <c r="G822" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="823" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A823" t="s">
         <v>336</v>
+      </c>
+      <c r="B823" t="s">
+        <v>335</v>
+      </c>
+      <c r="C823" t="s">
+        <v>217</v>
+      </c>
+      <c r="D823" t="s">
+        <v>218</v>
+      </c>
+      <c r="E823" t="s">
+        <v>350</v>
+      </c>
+      <c r="F823" t="s">
+        <v>338</v>
+      </c>
+      <c r="G823" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="824" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A824" t="s">
+        <v>336</v>
+      </c>
+      <c r="B824" t="s">
+        <v>335</v>
+      </c>
+      <c r="C824" t="s">
+        <v>199</v>
+      </c>
+      <c r="D824" t="s">
+        <v>200</v>
+      </c>
+      <c r="E824" t="s">
+        <v>350</v>
+      </c>
+      <c r="F824" t="s">
+        <v>338</v>
+      </c>
+      <c r="G824" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="825" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A825" t="s">
+        <v>336</v>
+      </c>
+      <c r="B825" t="s">
+        <v>335</v>
+      </c>
+      <c r="C825" t="s">
+        <v>213</v>
+      </c>
+      <c r="D825" t="s">
+        <v>214</v>
+      </c>
+      <c r="E825" t="s">
+        <v>350</v>
+      </c>
+      <c r="F825" t="s">
+        <v>338</v>
+      </c>
+      <c r="G825" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="826" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A826" t="s">
+        <v>336</v>
+      </c>
+      <c r="B826" t="s">
+        <v>335</v>
+      </c>
+      <c r="C826" t="s">
+        <v>343</v>
+      </c>
+      <c r="D826" t="s">
+        <v>344</v>
+      </c>
+      <c r="E826" t="s">
+        <v>350</v>
+      </c>
+      <c r="F826" t="s">
+        <v>338</v>
+      </c>
+      <c r="G826" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="827" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A827" t="s">
+        <v>336</v>
+      </c>
+      <c r="B827" t="s">
+        <v>335</v>
+      </c>
+      <c r="C827" t="s">
+        <v>345</v>
+      </c>
+      <c r="D827" t="s">
+        <v>346</v>
+      </c>
+      <c r="E827" t="s">
+        <v>350</v>
+      </c>
+      <c r="F827" t="s">
+        <v>338</v>
+      </c>
+      <c r="G827" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="828" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A828" t="s">
+        <v>336</v>
+      </c>
+      <c r="B828" t="s">
+        <v>335</v>
+      </c>
+      <c r="C828" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="D828" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="E828" t="s">
+        <v>350</v>
+      </c>
+      <c r="F828" t="s">
+        <v>338</v>
+      </c>
+      <c r="G828" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="829" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A829" t="s">
+        <v>336</v>
+      </c>
+      <c r="B829" t="s">
+        <v>335</v>
+      </c>
+      <c r="C829" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="D829" s="8" t="s">
+        <v>360</v>
+      </c>
+      <c r="E829" t="s">
+        <v>350</v>
+      </c>
+      <c r="F829" t="s">
+        <v>338</v>
+      </c>
+      <c r="G829" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="831" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A831" t="s">
+        <v>363</v>
+      </c>
+      <c r="B831" t="s">
+        <v>364</v>
+      </c>
+      <c r="C831" s="8" t="s">
+        <v>365</v>
+      </c>
+      <c r="D831" s="8" t="s">
+        <v>366</v>
+      </c>
+      <c r="E831" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="F831" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="832" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A832" t="s">
+        <v>363</v>
+      </c>
+      <c r="B832" t="s">
+        <v>364</v>
+      </c>
+      <c r="C832" t="s">
+        <v>368</v>
+      </c>
+      <c r="D832" t="s">
+        <v>369</v>
+      </c>
+      <c r="E832" t="s">
+        <v>350</v>
+      </c>
+      <c r="F832" t="s">
+        <v>338</v>
+      </c>
+      <c r="G832" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="833" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A833" t="s">
+        <v>363</v>
+      </c>
+      <c r="B833" t="s">
+        <v>364</v>
+      </c>
+      <c r="C833" t="s">
+        <v>317</v>
+      </c>
+      <c r="D833" t="s">
+        <v>318</v>
+      </c>
+      <c r="E833" t="s">
+        <v>350</v>
+      </c>
+      <c r="F833" t="s">
+        <v>338</v>
+      </c>
+      <c r="G833" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="834" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A834" t="s">
+        <v>363</v>
+      </c>
+      <c r="B834" t="s">
+        <v>364</v>
+      </c>
+      <c r="C834" t="s">
+        <v>372</v>
+      </c>
+      <c r="D834" t="s">
+        <v>373</v>
+      </c>
+      <c r="E834" t="s">
+        <v>350</v>
+      </c>
+      <c r="F834" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="835" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A835" t="s">
+        <v>363</v>
+      </c>
+      <c r="B835" t="s">
+        <v>364</v>
+      </c>
+      <c r="C835" t="s">
+        <v>374</v>
+      </c>
+      <c r="D835" t="s">
+        <v>375</v>
+      </c>
+      <c r="E835" t="s">
+        <v>350</v>
+      </c>
+      <c r="F835" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="836" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A836" t="s">
+        <v>363</v>
+      </c>
+      <c r="B836" t="s">
+        <v>364</v>
+      </c>
+      <c r="C836" t="s">
+        <v>376</v>
+      </c>
+      <c r="D836" t="s">
+        <v>377</v>
+      </c>
+      <c r="E836" t="s">
+        <v>350</v>
+      </c>
+      <c r="F836" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="837" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A837" t="s">
+        <v>363</v>
+      </c>
+      <c r="B837" t="s">
+        <v>364</v>
+      </c>
+      <c r="C837" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="D837" t="s">
+        <v>379</v>
+      </c>
+      <c r="E837" t="s">
+        <v>350</v>
+      </c>
+      <c r="F837" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="838" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A838" t="s">
+        <v>363</v>
+      </c>
+      <c r="B838" t="s">
+        <v>364</v>
+      </c>
+      <c r="C838" t="s">
+        <v>380</v>
+      </c>
+      <c r="D838" t="s">
+        <v>381</v>
+      </c>
+      <c r="E838" t="s">
+        <v>350</v>
+      </c>
+      <c r="F838" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="839" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A839" t="s">
+        <v>363</v>
+      </c>
+      <c r="B839" t="s">
+        <v>364</v>
+      </c>
+      <c r="C839" t="s">
+        <v>382</v>
+      </c>
+      <c r="D839" t="s">
+        <v>383</v>
+      </c>
+      <c r="E839" t="s">
+        <v>350</v>
+      </c>
+      <c r="F839" t="s">
+        <v>338</v>
       </c>
     </row>
   </sheetData>

</xml_diff>